<commit_message>
Leturer management: add hourly rating
</commit_message>
<xml_diff>
--- a/frontend/public/templates/recruitment_candidate_import_template.xlsx
+++ b/frontend/public/templates/recruitment_candidate_import_template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:H4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,18 +407,21 @@
         <v>email</v>
       </c>
       <c r="C1" t="str">
+        <v>Hourly Rate</v>
+      </c>
+      <c r="D1" t="str">
         <v>phone</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>positionAppliedFor</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>title</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>gender</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>interviewDate</v>
       </c>
     </row>
@@ -430,18 +433,21 @@
         <v>john.doe@cadt.edu.kh</v>
       </c>
       <c r="C2" t="str">
+        <v>12.50</v>
+      </c>
+      <c r="D2" t="str">
         <v>+85512345678</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>Lecturer</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>Mr</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>male</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>2026-03-25</v>
       </c>
     </row>
@@ -453,18 +459,21 @@
         <v>sokha.chan@cadt.edu.kh</v>
       </c>
       <c r="C3" t="str">
+        <v>18.00</v>
+      </c>
+      <c r="D3" t="str">
         <v>+85512987654</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>Advisor</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>Ms</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>female</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>2026-03-27</v>
       </c>
     </row>
@@ -476,24 +485,27 @@
         <v>dara.lim@cadt.edu.kh</v>
       </c>
       <c r="C4" t="str">
+        <v>9.75</v>
+      </c>
+      <c r="D4" t="str">
         <v>+85511999888</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>Teaching Assistant</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>Dr</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>other</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Modify contract summary, upload evaluation header
</commit_message>
<xml_diff>
--- a/frontend/public/templates/recruitment_candidate_import_template.xlsx
+++ b/frontend/public/templates/recruitment_candidate_import_template.xlsx
@@ -1,44 +1,145 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\YEAR3\TERM-2\CAPSTONE-2\lecturer-contract-management-system\frontend\public\templates\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93100E70-DACD-47D4-BF6A-F22BE6920389}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Candidates" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="34">
+  <si>
+    <t>fullName</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>Hourly Rate</t>
+  </si>
+  <si>
+    <t>phone</t>
+  </si>
+  <si>
+    <t>positionAppliedFor</t>
+  </si>
+  <si>
+    <t>title</t>
+  </si>
+  <si>
+    <t>gender</t>
+  </si>
+  <si>
+    <t>interviewDate</t>
+  </si>
+  <si>
+    <t>John Doe</t>
+  </si>
+  <si>
+    <t>john.doe@cadt.edu.kh</t>
+  </si>
+  <si>
+    <t>12.50</t>
+  </si>
+  <si>
+    <t>+85512345678</t>
+  </si>
+  <si>
+    <t>Lecturer</t>
+  </si>
+  <si>
+    <t>Mr</t>
+  </si>
+  <si>
+    <t>male</t>
+  </si>
+  <si>
+    <t>2026-03-25</t>
+  </si>
+  <si>
+    <t>Sokha Chan</t>
+  </si>
+  <si>
+    <t>sokha.chan@cadt.edu.kh</t>
+  </si>
+  <si>
+    <t>18.00</t>
+  </si>
+  <si>
+    <t>+85512987654</t>
+  </si>
+  <si>
+    <t>Advisor</t>
+  </si>
+  <si>
+    <t>Ms</t>
+  </si>
+  <si>
+    <t>female</t>
+  </si>
+  <si>
+    <t>2026-03-27</t>
+  </si>
+  <si>
+    <t>Dara Lim</t>
+  </si>
+  <si>
+    <t>dara.lim@cadt.edu.kh</t>
+  </si>
+  <si>
+    <t>9.75</t>
+  </si>
+  <si>
+    <t>+85511999888</t>
+  </si>
+  <si>
+    <t>Teaching Assistant</t>
+  </si>
+  <si>
+    <t>Dr</t>
+  </si>
+  <si>
+    <t>other</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Navid Kim</t>
+  </si>
+  <si>
+    <t>navid.kim@cadt.edu.kh</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -61,17 +162,28 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,116 +508,147 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="4" max="4" width="20.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>fullName</v>
-      </c>
-      <c r="B1" t="str">
-        <v>email</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Hourly Rate</v>
-      </c>
-      <c r="D1" t="str">
-        <v>phone</v>
-      </c>
-      <c r="E1" t="str">
-        <v>positionAppliedFor</v>
-      </c>
-      <c r="F1" t="str">
-        <v>title</v>
-      </c>
-      <c r="G1" t="str">
-        <v>gender</v>
-      </c>
-      <c r="H1" t="str">
-        <v>interviewDate</v>
+    <row r="1" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>John Doe</v>
-      </c>
-      <c r="B2" t="str">
-        <v>john.doe@cadt.edu.kh</v>
-      </c>
-      <c r="C2" t="str">
-        <v>12.50</v>
-      </c>
-      <c r="D2" t="str">
-        <v>+85512345678</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Lecturer</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Mr</v>
-      </c>
-      <c r="G2" t="str">
-        <v>male</v>
-      </c>
-      <c r="H2" t="str">
-        <v>2026-03-25</v>
+    <row r="2" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" t="s">
+        <v>15</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Sokha Chan</v>
-      </c>
-      <c r="B3" t="str">
-        <v>sokha.chan@cadt.edu.kh</v>
-      </c>
-      <c r="C3" t="str">
-        <v>18.00</v>
-      </c>
-      <c r="D3" t="str">
-        <v>+85512987654</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Advisor</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Ms</v>
-      </c>
-      <c r="G3" t="str">
-        <v>female</v>
-      </c>
-      <c r="H3" t="str">
-        <v>2026-03-27</v>
+    <row r="3" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" t="s">
+        <v>23</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Dara Lim</v>
-      </c>
-      <c r="B4" t="str">
-        <v>dara.lim@cadt.edu.kh</v>
-      </c>
-      <c r="C4" t="str">
-        <v>9.75</v>
-      </c>
-      <c r="D4" t="str">
-        <v>+85511999888</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Teaching Assistant</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Dr</v>
-      </c>
-      <c r="G4" t="str">
-        <v>other</v>
-      </c>
-      <c r="H4" t="str">
-        <v/>
+    <row r="4" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5">
+        <v>15</v>
+      </c>
+      <c r="D5">
+        <v>855732468234</v>
+      </c>
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B5" r:id="rId1" xr:uid="{43AAFDFC-F8CC-4EDA-BA34-3C6AD948E969}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
+    <ignoredError sqref="A1:H4" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>